<commit_message>
feat: migrate public cases to Home Credit 2018
Regenerate the seven public cases from the full application train/test inputs with deterministic whole-day partitions, null-label semantics, business metadata, native plots, and portable evidence. Update bilingual READMEs, docs, reproducibility checks, and CI; fix report denominators, stable ordering, long Excel metadata, and responsive rule tables.
</commit_message>
<xml_diff>
--- a/docs/assets/cases/correlation.xlsx
+++ b/docs/assets/cases/correlation.xlsx
@@ -14,18 +14,39 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="11">
   <si>
-    <t>main_score [主模型分; champion]</t>
+    <t>EXT_SOURCE_1 [外部来源分 1; Home Credit 2018 application_{train|test}.csv]</t>
   </si>
   <si>
-    <t>score_inverse [主分负向副本; champion]</t>
+    <t>EXT_SOURCE_2 [外部来源分 2; Home Credit 2018 application_{train|test}.csv]</t>
   </si>
   <si>
-    <t>income [申报月收入; application]</t>
+    <t>EXT_SOURCE_3 [外部来源分 3; Home Credit 2018 application_{train|test}.csv]</t>
   </si>
   <si>
-    <t>income_copy [收入冗余副本; application]</t>
+    <t>AMT_INCOME_TOTAL [客户收入; Home Credit 2018 application_{train|test}.csv]</t>
+  </si>
+  <si>
+    <t>AMT_ANNUITY [贷款年金; Home Credit 2018 application_{train|test}.csv]</t>
+  </si>
+  <si>
+    <t>AMT_GOODS_PRICE [贷款对应商品价格; Home Credit 2018 application_{train|test}.csv]</t>
+  </si>
+  <si>
+    <t>DAYS_BIRTH [申请时年龄天数（原始值）; Home Credit 2018 application_{train|test}.csv]</t>
+  </si>
+  <si>
+    <t>REGION_RATING_CLIENT [居住地区评级; Home Credit 2018 application_{train|test}.csv]</t>
+  </si>
+  <si>
+    <t>REGION_RATING_CLIENT_W_CITY [考虑城市的居住地区评级; Home Credit 2018 application_{train|test}.csv]</t>
+  </si>
+  <si>
+    <t>OBS_30_CNT_SOCIAL_CIRCLE [社交圈可观察的 30 天逾期记录数; Home Credit 2018 application_{train|test}.csv]</t>
+  </si>
+  <si>
+    <t>OBS_60_CNT_SOCIAL_CIRCLE [社交圈可观察的 60 天逾期记录数; Home Credit 2018 application_{train|test}.csv]</t>
   </si>
 </sst>
 </file>
@@ -55,7 +76,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="38">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -70,19 +91,211 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF053061"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF6F7F7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF7F6F6"/>
+        <fgColor rgb="FFFCD7C2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFDDDCB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF9EEE7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFAE8DE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCDFCF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4393C3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE1EDF3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEFF3F5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFAE7DC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFBE6DA"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFBE4D6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDEBF2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA7D0E4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA9D1E5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF0F4F6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE9F0F4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8F4F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8F1ED"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD2E6F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F6F7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEA8E70"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF3A481"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF3F5F6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCFE4EF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC7E0ED"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA81529"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE7F0F4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE0ECF3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDEEBF2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDAE9F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE6EFF4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE4EEF4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF7F5F4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF790622"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF9F0EB"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -99,12 +312,44 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="25" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="26" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="28" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="29" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="30" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="31" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="32" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="36" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="37" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -399,10 +644,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:12">
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -415,8 +660,29 @@
       <c r="E1" t="s">
         <v>3</v>
       </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:12">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -424,63 +690,413 @@
         <v>1</v>
       </c>
       <c r="C2" s="2">
-        <v>-1</v>
+        <v>0.215628947409865</v>
       </c>
       <c r="D2" s="3">
-        <v>-0.007641904253103273</v>
-      </c>
-      <c r="E2" s="3">
-        <v>-0.007641904253103273</v>
+        <v>0.1832839842557503</v>
+      </c>
+      <c r="E2" s="4">
+        <v>0.06347539823906737</v>
+      </c>
+      <c r="F2" s="5">
+        <v>0.1046555661873212</v>
+      </c>
+      <c r="G2" s="6">
+        <v>0.1643441611212416</v>
+      </c>
+      <c r="H2" s="7">
+        <v>-0.5983653685064243</v>
+      </c>
+      <c r="I2" s="8">
+        <v>-0.1098116017209118</v>
+      </c>
+      <c r="J2" s="8">
+        <v>-0.1098958927332886</v>
+      </c>
+      <c r="K2" s="9">
+        <v>-0.04243521348031969</v>
+      </c>
+      <c r="L2" s="9">
+        <v>-0.04218395668788743</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:12">
       <c r="A3" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="2">
-        <v>-1</v>
+        <v>0.215628947409865</v>
       </c>
       <c r="C3" s="1">
         <v>1</v>
       </c>
-      <c r="D3" s="4">
-        <v>0.007641904253103273</v>
-      </c>
-      <c r="E3" s="4">
-        <v>0.007641904253103273</v>
+      <c r="D3" s="10">
+        <v>0.1109876300160173</v>
+      </c>
+      <c r="E3" s="6">
+        <v>0.1674757372454293</v>
+      </c>
+      <c r="F3" s="11">
+        <v>0.119727887822526</v>
+      </c>
+      <c r="G3" s="12">
+        <v>0.1330003706488416</v>
+      </c>
+      <c r="H3" s="13">
+        <v>-0.1368893905158388</v>
+      </c>
+      <c r="I3" s="14">
+        <v>-0.3347520725461286</v>
+      </c>
+      <c r="J3" s="15">
+        <v>-0.3280024609246298</v>
+      </c>
+      <c r="K3" s="16">
+        <v>-0.0338434759222729</v>
+      </c>
+      <c r="L3" s="16">
+        <v>-0.03359079367805023</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:12">
       <c r="A4" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="3">
-        <v>-0.007641904253103273</v>
-      </c>
-      <c r="C4" s="4">
-        <v>0.007641904253103273</v>
+        <v>0.1832839842557503</v>
+      </c>
+      <c r="C4" s="10">
+        <v>0.1109876300160173</v>
       </c>
       <c r="D4" s="1">
         <v>1</v>
       </c>
-      <c r="E4" s="1">
-        <v>1</v>
+      <c r="E4" s="17">
+        <v>-0.07730138683592297</v>
+      </c>
+      <c r="F4" s="18">
+        <v>0.0210912215299875</v>
+      </c>
+      <c r="G4" s="19">
+        <v>0.04374953036483014</v>
+      </c>
+      <c r="H4" s="20">
+        <v>-0.1904399617131421</v>
+      </c>
+      <c r="I4" s="21">
+        <v>-0.008685130421744326</v>
+      </c>
+      <c r="J4" s="21">
+        <v>-0.009273429893834888</v>
+      </c>
+      <c r="K4" s="21">
+        <v>-0.009622225511633218</v>
+      </c>
+      <c r="L4" s="21">
+        <v>-0.009608193383749844</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:12">
       <c r="A5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="3">
-        <v>-0.007641904253103273</v>
-      </c>
-      <c r="C5" s="4">
-        <v>0.007641904253103273</v>
-      </c>
-      <c r="D5" s="1">
-        <v>1</v>
+      <c r="B5" s="4">
+        <v>0.06347539823906737</v>
+      </c>
+      <c r="C5" s="6">
+        <v>0.1674757372454293</v>
+      </c>
+      <c r="D5" s="17">
+        <v>-0.07730138683592297</v>
       </c>
       <c r="E5" s="1">
+        <v>1</v>
+      </c>
+      <c r="F5" s="22">
+        <v>0.4680234058290828</v>
+      </c>
+      <c r="G5" s="23">
+        <v>0.3985008600613512</v>
+      </c>
+      <c r="H5" s="24">
+        <v>-0.02016264816617007</v>
+      </c>
+      <c r="I5" s="25">
+        <v>-0.2084971790443018</v>
+      </c>
+      <c r="J5" s="26">
+        <v>-0.2286983475400514</v>
+      </c>
+      <c r="K5" s="9">
+        <v>-0.04528120673710537</v>
+      </c>
+      <c r="L5" s="9">
+        <v>-0.04512714325304314</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="5">
+        <v>0.1046555661873212</v>
+      </c>
+      <c r="C6" s="11">
+        <v>0.119727887822526</v>
+      </c>
+      <c r="D6" s="18">
+        <v>0.0210912215299875</v>
+      </c>
+      <c r="E6" s="22">
+        <v>0.4680234058290828</v>
+      </c>
+      <c r="F6" s="1">
+        <v>1</v>
+      </c>
+      <c r="G6" s="27">
+        <v>0.8243547988618424</v>
+      </c>
+      <c r="H6" s="28">
+        <v>-0.07886876491372243</v>
+      </c>
+      <c r="I6" s="29">
+        <v>-0.117653541137318</v>
+      </c>
+      <c r="J6" s="30">
+        <v>-0.1315608101237996</v>
+      </c>
+      <c r="K6" s="24">
+        <v>-0.02192713513732178</v>
+      </c>
+      <c r="L6" s="24">
+        <v>-0.02158707296064039</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="6">
+        <v>0.1643441611212416</v>
+      </c>
+      <c r="C7" s="12">
+        <v>0.1330003706488416</v>
+      </c>
+      <c r="D7" s="19">
+        <v>0.04374953036483014</v>
+      </c>
+      <c r="E7" s="23">
+        <v>0.3985008600613512</v>
+      </c>
+      <c r="F7" s="27">
+        <v>0.8243547988618424</v>
+      </c>
+      <c r="G7" s="1">
+        <v>1</v>
+      </c>
+      <c r="H7" s="31">
+        <v>-0.1519498627576819</v>
+      </c>
+      <c r="I7" s="32">
+        <v>-0.09065104883824958</v>
+      </c>
+      <c r="J7" s="33">
+        <v>-0.0995059696156303</v>
+      </c>
+      <c r="K7" s="21">
+        <v>-0.01088197109021203</v>
+      </c>
+      <c r="L7" s="21">
+        <v>-0.01067198989753664</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="7">
+        <v>-0.5983653685064243</v>
+      </c>
+      <c r="C8" s="13">
+        <v>-0.1368893905158388</v>
+      </c>
+      <c r="D8" s="20">
+        <v>-0.1904399617131421</v>
+      </c>
+      <c r="E8" s="24">
+        <v>-0.02016264816617007</v>
+      </c>
+      <c r="F8" s="28">
+        <v>-0.07886876491372243</v>
+      </c>
+      <c r="G8" s="31">
+        <v>-0.1519498627576819</v>
+      </c>
+      <c r="H8" s="1">
+        <v>1</v>
+      </c>
+      <c r="I8" s="34">
+        <v>0.01447258912132963</v>
+      </c>
+      <c r="J8" s="18">
+        <v>0.01620758247585651</v>
+      </c>
+      <c r="K8" s="19">
+        <v>0.04038715506644174</v>
+      </c>
+      <c r="L8" s="19">
+        <v>0.03992963704100433</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="8">
+        <v>-0.1098116017209118</v>
+      </c>
+      <c r="C9" s="14">
+        <v>-0.3347520725461286</v>
+      </c>
+      <c r="D9" s="21">
+        <v>-0.008685130421744326</v>
+      </c>
+      <c r="E9" s="25">
+        <v>-0.2084971790443018</v>
+      </c>
+      <c r="F9" s="29">
+        <v>-0.117653541137318</v>
+      </c>
+      <c r="G9" s="32">
+        <v>-0.09065104883824958</v>
+      </c>
+      <c r="H9" s="34">
+        <v>0.01447258912132963</v>
+      </c>
+      <c r="I9" s="1">
+        <v>1</v>
+      </c>
+      <c r="J9" s="35">
+        <v>0.9494694865950033</v>
+      </c>
+      <c r="K9" s="36">
+        <v>0.0506428281374878</v>
+      </c>
+      <c r="L9" s="36">
+        <v>0.05017910987999667</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="A10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="8">
+        <v>-0.1098958927332886</v>
+      </c>
+      <c r="C10" s="15">
+        <v>-0.3280024609246298</v>
+      </c>
+      <c r="D10" s="21">
+        <v>-0.009273429893834888</v>
+      </c>
+      <c r="E10" s="26">
+        <v>-0.2286983475400514</v>
+      </c>
+      <c r="F10" s="30">
+        <v>-0.1315608101237996</v>
+      </c>
+      <c r="G10" s="33">
+        <v>-0.0995059696156303</v>
+      </c>
+      <c r="H10" s="18">
+        <v>0.01620758247585651</v>
+      </c>
+      <c r="I10" s="35">
+        <v>0.9494694865950033</v>
+      </c>
+      <c r="J10" s="1">
+        <v>1</v>
+      </c>
+      <c r="K10" s="19">
+        <v>0.04678940234478736</v>
+      </c>
+      <c r="L10" s="19">
+        <v>0.04629401661578864</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="9">
+        <v>-0.04243521348031969</v>
+      </c>
+      <c r="C11" s="16">
+        <v>-0.0338434759222729</v>
+      </c>
+      <c r="D11" s="21">
+        <v>-0.009622225511633218</v>
+      </c>
+      <c r="E11" s="9">
+        <v>-0.04528120673710537</v>
+      </c>
+      <c r="F11" s="24">
+        <v>-0.02192713513732178</v>
+      </c>
+      <c r="G11" s="21">
+        <v>-0.01088197109021203</v>
+      </c>
+      <c r="H11" s="19">
+        <v>0.04038715506644174</v>
+      </c>
+      <c r="I11" s="36">
+        <v>0.0506428281374878</v>
+      </c>
+      <c r="J11" s="19">
+        <v>0.04678940234478736</v>
+      </c>
+      <c r="K11" s="1">
+        <v>1</v>
+      </c>
+      <c r="L11" s="1">
+        <v>0.9974968029828649</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="A12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="9">
+        <v>-0.04218395668788743</v>
+      </c>
+      <c r="C12" s="16">
+        <v>-0.03359079367805023</v>
+      </c>
+      <c r="D12" s="21">
+        <v>-0.009608193383749844</v>
+      </c>
+      <c r="E12" s="9">
+        <v>-0.04512714325304314</v>
+      </c>
+      <c r="F12" s="24">
+        <v>-0.02158707296064039</v>
+      </c>
+      <c r="G12" s="21">
+        <v>-0.01067198989753664</v>
+      </c>
+      <c r="H12" s="19">
+        <v>0.03992963704100433</v>
+      </c>
+      <c r="I12" s="36">
+        <v>0.05017910987999667</v>
+      </c>
+      <c r="J12" s="19">
+        <v>0.04629401661578864</v>
+      </c>
+      <c r="K12" s="1">
+        <v>0.9974968029828649</v>
+      </c>
+      <c r="L12" s="1">
         <v>1</v>
       </c>
     </row>

</xml_diff>